<commit_message>
Deploying to gh-pages from @ Sameerakhan05/pdd-testing@c6e2db39fa34b2fdaa4d4947b33aeda76e828364 🚀
</commit_message>
<xml_diff>
--- a/reports/history/build-5/Execution_Summary.xlsx
+++ b/reports/history/build-5/Execution_Summary.xlsx
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T07:18:14.131Z</t>
+    <t>2026-06-24T07:52:43.570Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>